<commit_message>
feat: adding script to convert canvas to images and download zip
</commit_message>
<xml_diff>
--- a/public/cards-template.xlsx
+++ b/public/cards-template.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="406">
   <si>
     <t>type</t>
   </si>
@@ -1259,7 +1259,7 @@
   </si>
   <si>
     <t>Players cannot Parry.
- &lt;B&gt;WEAK SPOT 2:&lt;/b&gt; This minion suffers 1
+ &lt;b&gt;WEAK SPOT 2:&lt;/b&gt; This minion suffers 1
  damage.
  Persistent: Lumière suffers 2 damage.</t>
   </si>
@@ -1760,7 +1760,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" ht="15.75" hidden="1" customHeight="1">
+    <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>24</v>
       </c>
@@ -1780,7 +1780,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="3" ht="15.75" hidden="1" customHeight="1">
+    <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>24</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>5.0</v>
       </c>
     </row>
-    <row r="4" ht="15.75" hidden="1" customHeight="1">
+    <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>24</v>
       </c>
@@ -1820,7 +1820,7 @@
         <v>5.0</v>
       </c>
     </row>
-    <row r="5" ht="15.75" hidden="1" customHeight="1">
+    <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="1" t="s">
         <v>24</v>
       </c>
@@ -1840,7 +1840,7 @@
         <v>6.0</v>
       </c>
     </row>
-    <row r="6" ht="15.75" hidden="1" customHeight="1">
+    <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
@@ -1860,7 +1860,7 @@
         <v>6.0</v>
       </c>
     </row>
-    <row r="7" ht="15.75" hidden="1" customHeight="1">
+    <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="1" t="s">
         <v>24</v>
       </c>
@@ -1880,7 +1880,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="8" ht="15.75" hidden="1" customHeight="1">
+    <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>24</v>
       </c>
@@ -1900,7 +1900,7 @@
         <v>5.0</v>
       </c>
     </row>
-    <row r="9" ht="15.75" hidden="1" customHeight="1">
+    <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
@@ -1920,7 +1920,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="10" ht="15.75" hidden="1" customHeight="1">
+    <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="1" t="s">
         <v>24</v>
       </c>
@@ -1940,7 +1940,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="11" ht="15.75" hidden="1" customHeight="1">
+    <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="1" t="s">
         <v>24</v>
       </c>
@@ -1960,7 +1960,7 @@
         <v>6.0</v>
       </c>
     </row>
-    <row r="12" ht="15.75" hidden="1" customHeight="1">
+    <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="1" t="s">
         <v>24</v>
       </c>
@@ -1980,7 +1980,7 @@
         <v>7.0</v>
       </c>
     </row>
-    <row r="13" ht="15.75" hidden="1" customHeight="1">
+    <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="1" t="s">
         <v>24</v>
       </c>
@@ -2000,7 +2000,7 @@
         <v>7.0</v>
       </c>
     </row>
-    <row r="14" ht="15.75" hidden="1" customHeight="1">
+    <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
@@ -2020,7 +2020,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="15" ht="15.75" hidden="1" customHeight="1">
+    <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="1" t="s">
         <v>24</v>
       </c>
@@ -2040,7 +2040,7 @@
         <v>5.0</v>
       </c>
     </row>
-    <row r="16" ht="15.75" hidden="1" customHeight="1">
+    <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="1" t="s">
         <v>24</v>
       </c>
@@ -2060,7 +2060,7 @@
         <v>8.0</v>
       </c>
     </row>
-    <row r="17" ht="15.75" hidden="1" customHeight="1">
+    <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="1" t="s">
         <v>24</v>
       </c>
@@ -2080,7 +2080,7 @@
         <v>6.0</v>
       </c>
     </row>
-    <row r="18" ht="15.75" hidden="1" customHeight="1">
+    <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="1" t="s">
         <v>24</v>
       </c>
@@ -2100,7 +2100,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="19" ht="15.75" hidden="1" customHeight="1">
+    <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="1" t="s">
         <v>24</v>
       </c>
@@ -2120,7 +2120,7 @@
         <v>5.0</v>
       </c>
     </row>
-    <row r="20" ht="15.75" hidden="1" customHeight="1">
+    <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="1" t="s">
         <v>24</v>
       </c>
@@ -2140,7 +2140,7 @@
         <v>7.0</v>
       </c>
     </row>
-    <row r="21" ht="15.75" hidden="1" customHeight="1">
+    <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="1" t="s">
         <v>24</v>
       </c>
@@ -2160,7 +2160,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="22" ht="15.75" hidden="1" customHeight="1">
+    <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="1" t="s">
         <v>72</v>
       </c>
@@ -2177,7 +2177,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="23" ht="15.75" hidden="1" customHeight="1">
+    <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="1" t="s">
         <v>72</v>
       </c>
@@ -2194,7 +2194,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="24" ht="15.75" hidden="1" customHeight="1">
+    <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="1" t="s">
         <v>72</v>
       </c>
@@ -2211,7 +2211,7 @@
         <v>5.0</v>
       </c>
     </row>
-    <row r="25" ht="15.75" hidden="1" customHeight="1">
+    <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="1" t="s">
         <v>72</v>
       </c>
@@ -2228,7 +2228,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="26" ht="15.75" hidden="1" customHeight="1">
+    <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="1" t="s">
         <v>72</v>
       </c>
@@ -2245,7 +2245,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="27" ht="15.75" hidden="1" customHeight="1">
+    <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="1" t="s">
         <v>72</v>
       </c>
@@ -2262,7 +2262,7 @@
         <v>5.0</v>
       </c>
     </row>
-    <row r="28" ht="15.75" hidden="1" customHeight="1">
+    <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="1" t="s">
         <v>85</v>
       </c>
@@ -2279,7 +2279,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="29" ht="15.75" hidden="1" customHeight="1">
+    <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="1" t="s">
         <v>85</v>
       </c>
@@ -2296,7 +2296,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="30" ht="15.75" hidden="1" customHeight="1">
+    <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="1" t="s">
         <v>85</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="31" ht="15.75" hidden="1" customHeight="1">
+    <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="1" t="s">
         <v>85</v>
       </c>
@@ -2330,7 +2330,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="32" ht="15.75" hidden="1" customHeight="1">
+    <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="1" t="s">
         <v>85</v>
       </c>
@@ -2347,7 +2347,7 @@
         <v>5.0</v>
       </c>
     </row>
-    <row r="33" ht="15.75" hidden="1" customHeight="1">
+    <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="1" t="s">
         <v>85</v>
       </c>
@@ -2374,6 +2374,9 @@
       <c r="C34" s="4" t="s">
         <v>100</v>
       </c>
+      <c r="E34" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="G34" s="4" t="s">
         <v>101</v>
       </c>
@@ -2394,6 +2397,9 @@
       <c r="C35" s="4" t="s">
         <v>103</v>
       </c>
+      <c r="E35" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="G35" s="4" t="s">
         <v>101</v>
       </c>
@@ -2414,6 +2420,9 @@
       <c r="C36" s="4" t="s">
         <v>105</v>
       </c>
+      <c r="E36" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="G36" s="4" t="s">
         <v>101</v>
       </c>
@@ -2424,7 +2433,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="37" ht="15.75" hidden="1" customHeight="1">
+    <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="2" t="s">
         <v>106</v>
       </c>
@@ -2441,7 +2450,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="38" ht="15.75" hidden="1" customHeight="1">
+    <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="2" t="s">
         <v>106</v>
       </c>
@@ -2458,7 +2467,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="39" ht="15.75" hidden="1" customHeight="1">
+    <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="2" t="s">
         <v>106</v>
       </c>
@@ -2475,7 +2484,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="40" ht="15.75" hidden="1" customHeight="1">
+    <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="2" t="s">
         <v>113</v>
       </c>
@@ -2492,7 +2501,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="41" ht="15.75" hidden="1" customHeight="1">
+    <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="2" t="s">
         <v>113</v>
       </c>
@@ -2509,7 +2518,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="42" ht="15.75" hidden="1" customHeight="1">
+    <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="2" t="s">
         <v>106</v>
       </c>
@@ -2526,7 +2535,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="43" ht="15.75" hidden="1" customHeight="1">
+    <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="2" t="s">
         <v>106</v>
       </c>
@@ -2543,7 +2552,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="44" ht="15.75" hidden="1" customHeight="1">
+    <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="2" t="s">
         <v>113</v>
       </c>
@@ -2560,7 +2569,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="45" ht="15.75" hidden="1" customHeight="1">
+    <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="2" t="s">
         <v>113</v>
       </c>
@@ -2577,7 +2586,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="46" ht="15.75" hidden="1" customHeight="1">
+    <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="2" t="s">
         <v>113</v>
       </c>
@@ -2604,6 +2613,9 @@
       <c r="C47" s="4" t="s">
         <v>129</v>
       </c>
+      <c r="E47" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="G47" s="4" t="s">
         <v>101</v>
       </c>
@@ -2624,6 +2636,9 @@
       <c r="C48" s="4" t="s">
         <v>131</v>
       </c>
+      <c r="E48" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="G48" s="4" t="s">
         <v>101</v>
       </c>
@@ -2634,7 +2649,7 @@
         <v>8.0</v>
       </c>
     </row>
-    <row r="49" ht="15.75" hidden="1" customHeight="1">
+    <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="2" t="s">
         <v>106</v>
       </c>
@@ -2651,7 +2666,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="50" ht="15.75" hidden="1" customHeight="1">
+    <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="2" t="s">
         <v>106</v>
       </c>
@@ -2668,7 +2683,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="51" ht="15.75" hidden="1" customHeight="1">
+    <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="2" t="s">
         <v>106</v>
       </c>
@@ -2685,7 +2700,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="52" ht="15.75" hidden="1" customHeight="1">
+    <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="2" t="s">
         <v>113</v>
       </c>
@@ -2702,7 +2717,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="53" ht="15.75" hidden="1" customHeight="1">
+    <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="2" t="s">
         <v>113</v>
       </c>
@@ -2729,6 +2744,9 @@
       <c r="C54" s="4" t="s">
         <v>143</v>
       </c>
+      <c r="E54" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="G54" s="4" t="s">
         <v>101</v>
       </c>
@@ -2749,6 +2767,9 @@
       <c r="C55" s="4" t="s">
         <v>145</v>
       </c>
+      <c r="E55" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="G55" s="4" t="s">
         <v>101</v>
       </c>
@@ -2759,7 +2780,7 @@
         <v>12.0</v>
       </c>
     </row>
-    <row r="56" ht="15.75" hidden="1" customHeight="1">
+    <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="2" t="s">
         <v>106</v>
       </c>
@@ -2776,7 +2797,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="57" ht="15.75" hidden="1" customHeight="1">
+    <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="2" t="s">
         <v>113</v>
       </c>
@@ -2803,6 +2824,9 @@
       <c r="C58" s="4" t="s">
         <v>151</v>
       </c>
+      <c r="E58" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="G58" s="4" t="s">
         <v>101</v>
       </c>
@@ -2813,7 +2837,7 @@
         <v>10.0</v>
       </c>
     </row>
-    <row r="59" ht="15.75" hidden="1" customHeight="1">
+    <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="2" t="s">
         <v>106</v>
       </c>
@@ -2830,7 +2854,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="60" ht="15.75" hidden="1" customHeight="1">
+    <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="2" t="s">
         <v>113</v>
       </c>
@@ -2847,7 +2871,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="61" ht="15.75" hidden="1" customHeight="1">
+    <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="2" t="s">
         <v>113</v>
       </c>
@@ -2874,6 +2898,9 @@
       <c r="C62" s="4" t="s">
         <v>159</v>
       </c>
+      <c r="E62" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="G62" s="4" t="s">
         <v>101</v>
       </c>
@@ -2894,6 +2921,9 @@
       <c r="C63" s="4" t="s">
         <v>161</v>
       </c>
+      <c r="E63" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="G63" s="4" t="s">
         <v>101</v>
       </c>
@@ -2904,7 +2934,7 @@
         <v>9.0</v>
       </c>
     </row>
-    <row r="64" ht="15.75" hidden="1" customHeight="1">
+    <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="2" t="s">
         <v>106</v>
       </c>
@@ -2921,7 +2951,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="65" ht="15.75" hidden="1" customHeight="1">
+    <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="2" t="s">
         <v>106</v>
       </c>
@@ -2938,7 +2968,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="66" ht="15.75" hidden="1" customHeight="1">
+    <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="2" t="s">
         <v>106</v>
       </c>
@@ -2955,7 +2985,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="67" ht="15.75" hidden="1" customHeight="1">
+    <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="2" t="s">
         <v>113</v>
       </c>
@@ -2972,7 +3002,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="68" ht="15.75" hidden="1" customHeight="1">
+    <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="2" t="s">
         <v>113</v>
       </c>
@@ -2999,6 +3029,9 @@
       <c r="C69" s="4" t="s">
         <v>173</v>
       </c>
+      <c r="E69" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="G69" s="4" t="s">
         <v>101</v>
       </c>
@@ -3019,6 +3052,9 @@
       <c r="C70" s="4" t="s">
         <v>175</v>
       </c>
+      <c r="E70" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="G70" s="4" t="s">
         <v>101</v>
       </c>
@@ -3029,7 +3065,7 @@
         <v>10.0</v>
       </c>
     </row>
-    <row r="71" ht="15.75" hidden="1" customHeight="1">
+    <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="4" t="s">
         <v>24</v>
       </c>
@@ -3046,7 +3082,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="72" ht="15.75" hidden="1" customHeight="1">
+    <row r="72" ht="15.75" customHeight="1">
       <c r="A72" s="4" t="s">
         <v>24</v>
       </c>
@@ -3063,7 +3099,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="73" ht="15.75" hidden="1" customHeight="1">
+    <row r="73" ht="15.75" customHeight="1">
       <c r="A73" s="4" t="s">
         <v>24</v>
       </c>
@@ -3080,7 +3116,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="74" ht="15.75" hidden="1" customHeight="1">
+    <row r="74" ht="15.75" customHeight="1">
       <c r="A74" s="4" t="s">
         <v>24</v>
       </c>
@@ -3097,7 +3133,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="75" ht="15.75" hidden="1" customHeight="1">
+    <row r="75" ht="15.75" customHeight="1">
       <c r="A75" s="4" t="s">
         <v>24</v>
       </c>
@@ -3114,7 +3150,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="76" ht="15.75" hidden="1" customHeight="1">
+    <row r="76" ht="15.75" customHeight="1">
       <c r="A76" s="4" t="s">
         <v>24</v>
       </c>
@@ -3131,7 +3167,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="77" ht="15.75" hidden="1" customHeight="1">
+    <row r="77" ht="15.75" customHeight="1">
       <c r="A77" s="4" t="s">
         <v>24</v>
       </c>
@@ -3148,7 +3184,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="78" ht="15.75" hidden="1" customHeight="1">
+    <row r="78" ht="15.75" customHeight="1">
       <c r="A78" s="4" t="s">
         <v>72</v>
       </c>
@@ -3165,7 +3201,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="79" ht="15.75" hidden="1" customHeight="1">
+    <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="4" t="s">
         <v>72</v>
       </c>
@@ -3182,7 +3218,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="80" ht="15.75" hidden="1" customHeight="1">
+    <row r="80" ht="15.75" customHeight="1">
       <c r="A80" s="4" t="s">
         <v>72</v>
       </c>
@@ -3199,7 +3235,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="81" ht="15.75" hidden="1" customHeight="1">
+    <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="4" t="s">
         <v>72</v>
       </c>
@@ -3216,7 +3252,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="82" ht="15.75" hidden="1" customHeight="1">
+    <row r="82" ht="15.75" customHeight="1">
       <c r="A82" s="4" t="s">
         <v>72</v>
       </c>
@@ -3233,7 +3269,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="83" ht="15.75" hidden="1" customHeight="1">
+    <row r="83" ht="15.75" customHeight="1">
       <c r="A83" s="4" t="s">
         <v>72</v>
       </c>
@@ -3250,7 +3286,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="84" ht="15.75" hidden="1" customHeight="1">
+    <row r="84" ht="15.75" customHeight="1">
       <c r="A84" s="4" t="s">
         <v>85</v>
       </c>
@@ -3264,7 +3300,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="85" ht="15.75" hidden="1" customHeight="1">
+    <row r="85" ht="15.75" customHeight="1">
       <c r="A85" s="4" t="s">
         <v>24</v>
       </c>
@@ -3281,7 +3317,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="86" ht="15.75" hidden="1" customHeight="1">
+    <row r="86" ht="15.75" customHeight="1">
       <c r="A86" s="4" t="s">
         <v>24</v>
       </c>
@@ -3298,7 +3334,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="87" ht="15.75" hidden="1" customHeight="1">
+    <row r="87" ht="15.75" customHeight="1">
       <c r="A87" s="4" t="s">
         <v>24</v>
       </c>
@@ -3315,7 +3351,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="88" ht="15.75" hidden="1" customHeight="1">
+    <row r="88" ht="15.75" customHeight="1">
       <c r="A88" s="4" t="s">
         <v>24</v>
       </c>
@@ -3332,7 +3368,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="89" ht="15.75" hidden="1" customHeight="1">
+    <row r="89" ht="15.75" customHeight="1">
       <c r="A89" s="4" t="s">
         <v>24</v>
       </c>
@@ -3349,7 +3385,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="90" ht="15.75" hidden="1" customHeight="1">
+    <row r="90" ht="15.75" customHeight="1">
       <c r="A90" s="4" t="s">
         <v>72</v>
       </c>
@@ -3366,7 +3402,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="91" ht="15.75" hidden="1" customHeight="1">
+    <row r="91" ht="15.75" customHeight="1">
       <c r="A91" s="4" t="s">
         <v>72</v>
       </c>
@@ -3383,7 +3419,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="92" ht="15.75" hidden="1" customHeight="1">
+    <row r="92" ht="15.75" customHeight="1">
       <c r="A92" s="4" t="s">
         <v>72</v>
       </c>
@@ -3400,7 +3436,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="93" ht="15.75" hidden="1" customHeight="1">
+    <row r="93" ht="15.75" customHeight="1">
       <c r="A93" s="4" t="s">
         <v>72</v>
       </c>
@@ -3417,7 +3453,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="94" ht="15.75" hidden="1" customHeight="1">
+    <row r="94" ht="15.75" customHeight="1">
       <c r="A94" s="4" t="s">
         <v>72</v>
       </c>
@@ -3434,7 +3470,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="95" ht="15.75" hidden="1" customHeight="1">
+    <row r="95" ht="15.75" customHeight="1">
       <c r="A95" s="4" t="s">
         <v>72</v>
       </c>
@@ -3451,7 +3487,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="96" ht="15.75" hidden="1" customHeight="1">
+    <row r="96" ht="15.75" customHeight="1">
       <c r="A96" s="4" t="s">
         <v>72</v>
       </c>
@@ -3468,7 +3504,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="97" ht="15.75" hidden="1" customHeight="1">
+    <row r="97" ht="15.75" customHeight="1">
       <c r="A97" s="4" t="s">
         <v>72</v>
       </c>
@@ -3485,7 +3521,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="98" ht="15.75" hidden="1" customHeight="1">
+    <row r="98" ht="15.75" customHeight="1">
       <c r="A98" s="4" t="s">
         <v>72</v>
       </c>
@@ -3502,7 +3538,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="99" ht="15.75" hidden="1" customHeight="1">
+    <row r="99" ht="15.75" customHeight="1">
       <c r="A99" s="4" t="s">
         <v>72</v>
       </c>
@@ -3519,7 +3555,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="100" ht="15.75" hidden="1" customHeight="1">
+    <row r="100" ht="15.75" customHeight="1">
       <c r="A100" s="4" t="s">
         <v>72</v>
       </c>
@@ -3536,7 +3572,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="101" ht="15.75" hidden="1" customHeight="1">
+    <row r="101" ht="15.75" customHeight="1">
       <c r="A101" s="4" t="s">
         <v>72</v>
       </c>
@@ -3553,7 +3589,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="102" ht="15.75" hidden="1" customHeight="1">
+    <row r="102" ht="15.75" customHeight="1">
       <c r="A102" s="4" t="s">
         <v>72</v>
       </c>
@@ -3570,7 +3606,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="103" ht="15.75" hidden="1" customHeight="1">
+    <row r="103" ht="15.75" customHeight="1">
       <c r="A103" s="4" t="s">
         <v>72</v>
       </c>
@@ -3587,7 +3623,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="104" ht="15.75" hidden="1" customHeight="1">
+    <row r="104" ht="15.75" customHeight="1">
       <c r="A104" s="4" t="s">
         <v>72</v>
       </c>
@@ -3604,7 +3640,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="105" ht="15.75" hidden="1" customHeight="1">
+    <row r="105" ht="15.75" customHeight="1">
       <c r="A105" s="4" t="s">
         <v>72</v>
       </c>
@@ -3621,7 +3657,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="106" ht="15.75" hidden="1" customHeight="1">
+    <row r="106" ht="15.75" customHeight="1">
       <c r="A106" s="4" t="s">
         <v>72</v>
       </c>
@@ -3638,7 +3674,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="107" ht="15.75" hidden="1" customHeight="1">
+    <row r="107" ht="15.75" customHeight="1">
       <c r="A107" s="4" t="s">
         <v>72</v>
       </c>
@@ -3655,7 +3691,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="108" ht="15.75" hidden="1" customHeight="1">
+    <row r="108" ht="15.75" customHeight="1">
       <c r="A108" s="4" t="s">
         <v>72</v>
       </c>
@@ -3672,7 +3708,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="109" ht="15.75" hidden="1" customHeight="1">
+    <row r="109" ht="15.75" customHeight="1">
       <c r="A109" s="4" t="s">
         <v>72</v>
       </c>
@@ -3689,7 +3725,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="110" ht="15.75" hidden="1" customHeight="1">
+    <row r="110" ht="15.75" customHeight="1">
       <c r="A110" s="4" t="s">
         <v>72</v>
       </c>
@@ -3706,7 +3742,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="111" ht="15.75" hidden="1" customHeight="1">
+    <row r="111" ht="15.75" customHeight="1">
       <c r="A111" s="4" t="s">
         <v>72</v>
       </c>
@@ -3723,7 +3759,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="112" ht="15.75" hidden="1" customHeight="1">
+    <row r="112" ht="15.75" customHeight="1">
       <c r="A112" s="4" t="s">
         <v>72</v>
       </c>
@@ -3740,7 +3776,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="113" ht="15.75" hidden="1" customHeight="1">
+    <row r="113" ht="15.75" customHeight="1">
       <c r="A113" s="4" t="s">
         <v>72</v>
       </c>
@@ -3757,7 +3793,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="114" ht="15.75" hidden="1" customHeight="1">
+    <row r="114" ht="15.75" customHeight="1">
       <c r="A114" s="2" t="s">
         <v>106</v>
       </c>
@@ -3797,7 +3833,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="116" ht="15.75" hidden="1" customHeight="1">
+    <row r="116" ht="15.75" customHeight="1">
       <c r="A116" s="2" t="s">
         <v>113</v>
       </c>
@@ -3814,7 +3850,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="117" ht="15.75" hidden="1" customHeight="1">
+    <row r="117" ht="15.75" customHeight="1">
       <c r="A117" s="2" t="s">
         <v>113</v>
       </c>
@@ -3854,7 +3890,7 @@
         <v>5.0</v>
       </c>
     </row>
-    <row r="119" ht="15.75" hidden="1" customHeight="1">
+    <row r="119" ht="15.75" customHeight="1">
       <c r="A119" s="2" t="s">
         <v>113</v>
       </c>
@@ -3871,7 +3907,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="120" ht="15.75" hidden="1" customHeight="1">
+    <row r="120" ht="15.75" customHeight="1">
       <c r="A120" s="2" t="s">
         <v>113</v>
       </c>
@@ -3911,7 +3947,7 @@
         <v>12.0</v>
       </c>
     </row>
-    <row r="122" ht="15.75" hidden="1" customHeight="1">
+    <row r="122" ht="15.75" customHeight="1">
       <c r="A122" s="2" t="s">
         <v>106</v>
       </c>
@@ -3928,7 +3964,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="123" ht="15.75" hidden="1" customHeight="1">
+    <row r="123" ht="15.75" customHeight="1">
       <c r="A123" s="2" t="s">
         <v>106</v>
       </c>
@@ -3945,7 +3981,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="124" ht="15.75" hidden="1" customHeight="1">
+    <row r="124" ht="15.75" customHeight="1">
       <c r="A124" s="2" t="s">
         <v>106</v>
       </c>
@@ -3985,7 +4021,7 @@
         <v>8.0</v>
       </c>
     </row>
-    <row r="126" ht="15.75" hidden="1" customHeight="1">
+    <row r="126" ht="15.75" customHeight="1">
       <c r="A126" s="2" t="s">
         <v>113</v>
       </c>
@@ -4025,7 +4061,7 @@
         <v>10.0</v>
       </c>
     </row>
-    <row r="128" ht="15.75" hidden="1" customHeight="1">
+    <row r="128" ht="15.75" customHeight="1">
       <c r="A128" s="2" t="s">
         <v>106</v>
       </c>
@@ -4065,7 +4101,7 @@
         <v>12.0</v>
       </c>
     </row>
-    <row r="130" ht="15.75" hidden="1" customHeight="1">
+    <row r="130" ht="15.75" customHeight="1">
       <c r="A130" s="2" t="s">
         <v>113</v>
       </c>
@@ -4082,7 +4118,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="131" ht="15.75" hidden="1" customHeight="1">
+    <row r="131" ht="15.75" customHeight="1">
       <c r="A131" s="2" t="s">
         <v>106</v>
       </c>
@@ -4260,7 +4296,7 @@
         <v>5.0</v>
       </c>
     </row>
-    <row r="139" ht="15.75" hidden="1" customHeight="1">
+    <row r="139" ht="15.75" customHeight="1">
       <c r="A139" s="2" t="s">
         <v>113</v>
       </c>
@@ -4346,7 +4382,7 @@
         <v>6.0</v>
       </c>
     </row>
-    <row r="143" ht="15.75" hidden="1" customHeight="1">
+    <row r="143" ht="15.75" customHeight="1">
       <c r="A143" s="2" t="s">
         <v>113</v>
       </c>
@@ -4363,7 +4399,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="144" ht="15.75" hidden="1" customHeight="1">
+    <row r="144" ht="15.75" customHeight="1">
       <c r="A144" s="2" t="s">
         <v>106</v>
       </c>
@@ -4380,7 +4416,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="145" ht="15.75" hidden="1" customHeight="1">
+    <row r="145" ht="15.75" customHeight="1">
       <c r="A145" s="2" t="s">
         <v>113</v>
       </c>
@@ -4443,7 +4479,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="148" ht="15.75" hidden="1" customHeight="1">
+    <row r="148" ht="15.75" customHeight="1">
       <c r="A148" s="2" t="s">
         <v>106</v>
       </c>
@@ -4483,7 +4519,7 @@
         <v>9.0</v>
       </c>
     </row>
-    <row r="150" ht="15.75" hidden="1" customHeight="1">
+    <row r="150" ht="15.75" customHeight="1">
       <c r="A150" s="2" t="s">
         <v>106</v>
       </c>
@@ -4546,7 +4582,7 @@
         <v>12.0</v>
       </c>
     </row>
-    <row r="153" ht="15.75" hidden="1" customHeight="1">
+    <row r="153" ht="15.75" customHeight="1">
       <c r="A153" s="2" t="s">
         <v>113</v>
       </c>
@@ -4563,7 +4599,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="154" ht="15.75" hidden="1" customHeight="1">
+    <row r="154" ht="15.75" customHeight="1">
       <c r="A154" s="2" t="s">
         <v>106</v>
       </c>
@@ -4603,7 +4639,7 @@
         <v>10.0</v>
       </c>
     </row>
-    <row r="156" ht="15.75" hidden="1" customHeight="1">
+    <row r="156" ht="15.75" customHeight="1">
       <c r="A156" s="2" t="s">
         <v>106</v>
       </c>
@@ -4620,7 +4656,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="157" ht="15.75" hidden="1" customHeight="1">
+    <row r="157" ht="15.75" customHeight="1">
       <c r="A157" s="2" t="s">
         <v>106</v>
       </c>
@@ -4637,7 +4673,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="158" ht="15.75" hidden="1" customHeight="1">
+    <row r="158" ht="15.75" customHeight="1">
       <c r="A158" s="2" t="s">
         <v>113</v>
       </c>
@@ -4700,7 +4736,7 @@
         <v>9.0</v>
       </c>
     </row>
-    <row r="161" ht="15.75" hidden="1" customHeight="1">
+    <row r="161" ht="15.75" customHeight="1">
       <c r="A161" s="2" t="s">
         <v>106</v>
       </c>
@@ -4740,7 +4776,7 @@
         <v>14.0</v>
       </c>
     </row>
-    <row r="163" ht="15.75" hidden="1" customHeight="1">
+    <row r="163" ht="15.75" customHeight="1">
       <c r="A163" s="2" t="s">
         <v>113</v>
       </c>
@@ -4757,7 +4793,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="164" ht="15.75" hidden="1" customHeight="1">
+    <row r="164" ht="15.75" customHeight="1">
       <c r="A164" s="2" t="s">
         <v>113</v>
       </c>
@@ -4774,7 +4810,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="165" ht="15.75" hidden="1" customHeight="1">
+    <row r="165" ht="15.75" customHeight="1">
       <c r="A165" s="2" t="s">
         <v>106</v>
       </c>
@@ -4814,7 +4850,7 @@
         <v>8.0</v>
       </c>
     </row>
-    <row r="167" ht="15.75" hidden="1" customHeight="1">
+    <row r="167" ht="15.75" customHeight="1">
       <c r="A167" s="2" t="s">
         <v>113</v>
       </c>
@@ -4838,7 +4874,7 @@
       <c r="B168" s="4" t="s">
         <v>365</v>
       </c>
-      <c r="C168" s="4" t="s">
+      <c r="C168" s="5" t="s">
         <v>366</v>
       </c>
       <c r="E168" s="3" t="s">
@@ -4854,7 +4890,7 @@
         <v>13.0</v>
       </c>
     </row>
-    <row r="169" ht="15.75" hidden="1" customHeight="1">
+    <row r="169" ht="15.75" customHeight="1">
       <c r="A169" s="2" t="s">
         <v>106</v>
       </c>
@@ -4894,7 +4930,7 @@
         <v>18.0</v>
       </c>
     </row>
-    <row r="171" ht="15.75" hidden="1" customHeight="1">
+    <row r="171" ht="15.75" customHeight="1">
       <c r="A171" s="2" t="s">
         <v>113</v>
       </c>
@@ -4911,7 +4947,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="172" ht="15.75" hidden="1" customHeight="1">
+    <row r="172" ht="15.75" customHeight="1">
       <c r="A172" s="2" t="s">
         <v>106</v>
       </c>
@@ -4928,7 +4964,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="173" ht="15.75" hidden="1" customHeight="1">
+    <row r="173" ht="15.75" customHeight="1">
       <c r="A173" s="5" t="s">
         <v>6</v>
       </c>
@@ -4957,7 +4993,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="174" ht="15.75" hidden="1" customHeight="1">
+    <row r="174" ht="15.75" customHeight="1">
       <c r="A174" s="5" t="s">
         <v>6</v>
       </c>
@@ -4986,7 +5022,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="175" ht="15.75" hidden="1" customHeight="1">
+    <row r="175" ht="15.75" customHeight="1">
       <c r="A175" s="5" t="s">
         <v>6</v>
       </c>
@@ -5015,7 +5051,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="176" ht="15.75" hidden="1" customHeight="1">
+    <row r="176" ht="15.75" customHeight="1">
       <c r="A176" s="5" t="s">
         <v>6</v>
       </c>
@@ -5044,7 +5080,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="177" ht="15.75" hidden="1" customHeight="1">
+    <row r="177" ht="15.75" customHeight="1">
       <c r="A177" s="5" t="s">
         <v>6</v>
       </c>
@@ -5073,7 +5109,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="178" ht="15.75" hidden="1" customHeight="1">
+    <row r="178" ht="15.75" customHeight="1">
       <c r="A178" s="5" t="s">
         <v>6</v>
       </c>
@@ -5880,13 +5916,7 @@
     <row r="954" ht="15.75" customHeight="1"/>
     <row r="955" ht="15.75" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="$A$1:$X$178">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="minion"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="$A$1:$X$178"/>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="E2"/>
     <hyperlink r:id="rId2" ref="E3"/>
@@ -5920,78 +5950,90 @@
     <hyperlink r:id="rId30" ref="E31"/>
     <hyperlink r:id="rId31" ref="E32"/>
     <hyperlink r:id="rId32" ref="E33"/>
-    <hyperlink r:id="rId33" ref="E71"/>
-    <hyperlink r:id="rId34" ref="E72"/>
-    <hyperlink r:id="rId35" ref="E73"/>
-    <hyperlink r:id="rId36" ref="E74"/>
-    <hyperlink r:id="rId37" ref="E75"/>
-    <hyperlink r:id="rId38" ref="E76"/>
-    <hyperlink r:id="rId39" ref="E77"/>
-    <hyperlink r:id="rId40" ref="E78"/>
-    <hyperlink r:id="rId41" ref="E79"/>
-    <hyperlink r:id="rId42" ref="E80"/>
-    <hyperlink r:id="rId43" ref="E81"/>
-    <hyperlink r:id="rId44" ref="E82"/>
-    <hyperlink r:id="rId45" ref="E83"/>
-    <hyperlink r:id="rId46" ref="E84"/>
-    <hyperlink r:id="rId47" ref="E85"/>
-    <hyperlink r:id="rId48" ref="E86"/>
-    <hyperlink r:id="rId49" ref="E87"/>
-    <hyperlink r:id="rId50" ref="E88"/>
-    <hyperlink r:id="rId51" ref="E89"/>
-    <hyperlink r:id="rId52" ref="E90"/>
-    <hyperlink r:id="rId53" ref="E91"/>
-    <hyperlink r:id="rId54" ref="E92"/>
-    <hyperlink r:id="rId55" ref="E93"/>
-    <hyperlink r:id="rId56" ref="E94"/>
-    <hyperlink r:id="rId57" ref="E95"/>
-    <hyperlink r:id="rId58" ref="E96"/>
-    <hyperlink r:id="rId59" ref="E97"/>
-    <hyperlink r:id="rId60" ref="E98"/>
-    <hyperlink r:id="rId61" ref="E99"/>
-    <hyperlink r:id="rId62" ref="E100"/>
-    <hyperlink r:id="rId63" ref="E101"/>
-    <hyperlink r:id="rId64" ref="E102"/>
-    <hyperlink r:id="rId65" ref="E103"/>
-    <hyperlink r:id="rId66" ref="E104"/>
-    <hyperlink r:id="rId67" ref="E105"/>
-    <hyperlink r:id="rId68" ref="E106"/>
-    <hyperlink r:id="rId69" ref="E107"/>
-    <hyperlink r:id="rId70" ref="E108"/>
-    <hyperlink r:id="rId71" ref="E109"/>
-    <hyperlink r:id="rId72" ref="E110"/>
-    <hyperlink r:id="rId73" ref="E111"/>
-    <hyperlink r:id="rId74" ref="E112"/>
-    <hyperlink r:id="rId75" ref="E113"/>
-    <hyperlink r:id="rId76" ref="E115"/>
-    <hyperlink r:id="rId77" ref="E118"/>
-    <hyperlink r:id="rId78" ref="E121"/>
-    <hyperlink r:id="rId79" ref="E125"/>
-    <hyperlink r:id="rId80" ref="E127"/>
-    <hyperlink r:id="rId81" ref="E129"/>
-    <hyperlink r:id="rId82" ref="E132"/>
-    <hyperlink r:id="rId83" ref="E133"/>
-    <hyperlink r:id="rId84" ref="E134"/>
-    <hyperlink r:id="rId85" ref="E135"/>
-    <hyperlink r:id="rId86" ref="E136"/>
-    <hyperlink r:id="rId87" ref="E137"/>
-    <hyperlink r:id="rId88" ref="E138"/>
-    <hyperlink r:id="rId89" ref="E140"/>
-    <hyperlink r:id="rId90" ref="E141"/>
-    <hyperlink r:id="rId91" ref="E142"/>
-    <hyperlink r:id="rId92" ref="E146"/>
-    <hyperlink r:id="rId93" ref="E147"/>
-    <hyperlink r:id="rId94" ref="E149"/>
-    <hyperlink r:id="rId95" ref="E151"/>
-    <hyperlink r:id="rId96" ref="E152"/>
-    <hyperlink r:id="rId97" ref="E155"/>
-    <hyperlink r:id="rId98" ref="E159"/>
-    <hyperlink r:id="rId99" ref="E160"/>
-    <hyperlink r:id="rId100" ref="E162"/>
-    <hyperlink r:id="rId101" ref="E166"/>
-    <hyperlink r:id="rId102" ref="E168"/>
-    <hyperlink r:id="rId103" ref="E170"/>
+    <hyperlink r:id="rId33" ref="E34"/>
+    <hyperlink r:id="rId34" ref="E35"/>
+    <hyperlink r:id="rId35" ref="E36"/>
+    <hyperlink r:id="rId36" ref="E47"/>
+    <hyperlink r:id="rId37" ref="E48"/>
+    <hyperlink r:id="rId38" ref="E54"/>
+    <hyperlink r:id="rId39" ref="E55"/>
+    <hyperlink r:id="rId40" ref="E58"/>
+    <hyperlink r:id="rId41" ref="E62"/>
+    <hyperlink r:id="rId42" ref="E63"/>
+    <hyperlink r:id="rId43" ref="E69"/>
+    <hyperlink r:id="rId44" ref="E70"/>
+    <hyperlink r:id="rId45" ref="E71"/>
+    <hyperlink r:id="rId46" ref="E72"/>
+    <hyperlink r:id="rId47" ref="E73"/>
+    <hyperlink r:id="rId48" ref="E74"/>
+    <hyperlink r:id="rId49" ref="E75"/>
+    <hyperlink r:id="rId50" ref="E76"/>
+    <hyperlink r:id="rId51" ref="E77"/>
+    <hyperlink r:id="rId52" ref="E78"/>
+    <hyperlink r:id="rId53" ref="E79"/>
+    <hyperlink r:id="rId54" ref="E80"/>
+    <hyperlink r:id="rId55" ref="E81"/>
+    <hyperlink r:id="rId56" ref="E82"/>
+    <hyperlink r:id="rId57" ref="E83"/>
+    <hyperlink r:id="rId58" ref="E84"/>
+    <hyperlink r:id="rId59" ref="E85"/>
+    <hyperlink r:id="rId60" ref="E86"/>
+    <hyperlink r:id="rId61" ref="E87"/>
+    <hyperlink r:id="rId62" ref="E88"/>
+    <hyperlink r:id="rId63" ref="E89"/>
+    <hyperlink r:id="rId64" ref="E90"/>
+    <hyperlink r:id="rId65" ref="E91"/>
+    <hyperlink r:id="rId66" ref="E92"/>
+    <hyperlink r:id="rId67" ref="E93"/>
+    <hyperlink r:id="rId68" ref="E94"/>
+    <hyperlink r:id="rId69" ref="E95"/>
+    <hyperlink r:id="rId70" ref="E96"/>
+    <hyperlink r:id="rId71" ref="E97"/>
+    <hyperlink r:id="rId72" ref="E98"/>
+    <hyperlink r:id="rId73" ref="E99"/>
+    <hyperlink r:id="rId74" ref="E100"/>
+    <hyperlink r:id="rId75" ref="E101"/>
+    <hyperlink r:id="rId76" ref="E102"/>
+    <hyperlink r:id="rId77" ref="E103"/>
+    <hyperlink r:id="rId78" ref="E104"/>
+    <hyperlink r:id="rId79" ref="E105"/>
+    <hyperlink r:id="rId80" ref="E106"/>
+    <hyperlink r:id="rId81" ref="E107"/>
+    <hyperlink r:id="rId82" ref="E108"/>
+    <hyperlink r:id="rId83" ref="E109"/>
+    <hyperlink r:id="rId84" ref="E110"/>
+    <hyperlink r:id="rId85" ref="E111"/>
+    <hyperlink r:id="rId86" ref="E112"/>
+    <hyperlink r:id="rId87" ref="E113"/>
+    <hyperlink r:id="rId88" ref="E115"/>
+    <hyperlink r:id="rId89" ref="E118"/>
+    <hyperlink r:id="rId90" ref="E121"/>
+    <hyperlink r:id="rId91" ref="E125"/>
+    <hyperlink r:id="rId92" ref="E127"/>
+    <hyperlink r:id="rId93" ref="E129"/>
+    <hyperlink r:id="rId94" ref="E132"/>
+    <hyperlink r:id="rId95" ref="E133"/>
+    <hyperlink r:id="rId96" ref="E134"/>
+    <hyperlink r:id="rId97" ref="E135"/>
+    <hyperlink r:id="rId98" ref="E136"/>
+    <hyperlink r:id="rId99" ref="E137"/>
+    <hyperlink r:id="rId100" ref="E138"/>
+    <hyperlink r:id="rId101" ref="E140"/>
+    <hyperlink r:id="rId102" ref="E141"/>
+    <hyperlink r:id="rId103" ref="E142"/>
+    <hyperlink r:id="rId104" ref="E146"/>
+    <hyperlink r:id="rId105" ref="E147"/>
+    <hyperlink r:id="rId106" ref="E149"/>
+    <hyperlink r:id="rId107" ref="E151"/>
+    <hyperlink r:id="rId108" ref="E152"/>
+    <hyperlink r:id="rId109" ref="E155"/>
+    <hyperlink r:id="rId110" ref="E159"/>
+    <hyperlink r:id="rId111" ref="E160"/>
+    <hyperlink r:id="rId112" ref="E162"/>
+    <hyperlink r:id="rId113" ref="E166"/>
+    <hyperlink r:id="rId114" ref="E168"/>
+    <hyperlink r:id="rId115" ref="E170"/>
   </hyperlinks>
-  <drawing r:id="rId104"/>
+  <drawing r:id="rId116"/>
 </worksheet>
 </file>
</xml_diff>